<commit_message>
Complete search location functionality
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Datadriven-OrangeHrm.xlsx
+++ b/src/test/resources/data/Datadriven-OrangeHrm.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Studying\GraduateProject\orangehrmtesting\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB41761-0346-46A8-B750-9C3021343552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7105961-19E8-4AC7-9509-C1F14B6D6003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{25C74C23-6D17-4E04-9252-4B94296A7369}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{25C74C23-6D17-4E04-9252-4B94296A7369}"/>
   </bookViews>
   <sheets>
     <sheet name="loginFail" sheetId="1" r:id="rId1"/>
     <sheet name="Search" sheetId="2" r:id="rId2"/>
+    <sheet name="Search Location" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
   <si>
     <t>Username</t>
   </si>
@@ -88,6 +89,27 @@
   </si>
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>Đống Đa</t>
+  </si>
+  <si>
+    <t>Hà Nội</t>
+  </si>
+  <si>
+    <t>Viet Nam</t>
   </si>
 </sst>
 </file>
@@ -580,4 +602,46 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F35673-FDC9-419A-9CAF-7B580C323A56}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Complete PIM Tab and currently developing the remaining three tabs
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Datadriven-OrangeHrm.xlsx
+++ b/src/test/resources/data/Datadriven-OrangeHrm.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Studying\GraduateProject\orangehrmtesting\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7105961-19E8-4AC7-9509-C1F14B6D6003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA268A4-C1DD-4F41-A201-BC2C91B25105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{25C74C23-6D17-4E04-9252-4B94296A7369}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{25C74C23-6D17-4E04-9252-4B94296A7369}"/>
   </bookViews>
   <sheets>
     <sheet name="loginFail" sheetId="1" r:id="rId1"/>
     <sheet name="Search" sheetId="2" r:id="rId2"/>
     <sheet name="Search Location" sheetId="3" r:id="rId3"/>
+    <sheet name="Employee" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
   <si>
     <t>Username</t>
   </si>
@@ -110,16 +111,65 @@
   </si>
   <si>
     <t>Viet Nam</t>
+  </si>
+  <si>
+    <t>Supervisor Name</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Employement Status</t>
+  </si>
+  <si>
+    <t>Include</t>
+  </si>
+  <si>
+    <t>Job Title</t>
+  </si>
+  <si>
+    <t>Sub Unit</t>
+  </si>
+  <si>
+    <t>Huy Deliver</t>
+  </si>
+  <si>
+    <t>Nguyễn Huy Bách</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>Full Time Contract</t>
+  </si>
+  <si>
+    <t>Current Employees Only</t>
+  </si>
+  <si>
+    <t>Devops</t>
+  </si>
+  <si>
+    <t>OrangeHRM</t>
+  </si>
+  <si>
+    <t>Current and Past Employees</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
@@ -644,4 +694,87 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF2A67B0-D40E-47CE-8D8C-FABDD5073471}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.8984375" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" customWidth="1"/>
+    <col min="4" max="4" width="24.19921875" customWidth="1"/>
+    <col min="5" max="5" width="24.296875" customWidth="1"/>
+    <col min="7" max="7" width="19.296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Complete CRUD vacancy of Recruitment
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Datadriven-OrangeHrm.xlsx
+++ b/src/test/resources/data/Datadriven-OrangeHrm.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Studying\GraduateProject\orangehrmtesting\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA268A4-C1DD-4F41-A201-BC2C91B25105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23494EE-93CB-48CF-8401-B6C9CA3B5C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{25C74C23-6D17-4E04-9252-4B94296A7369}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{25C74C23-6D17-4E04-9252-4B94296A7369}"/>
   </bookViews>
   <sheets>
     <sheet name="loginFail" sheetId="1" r:id="rId1"/>
     <sheet name="Search" sheetId="2" r:id="rId2"/>
     <sheet name="Search Location" sheetId="3" r:id="rId3"/>
     <sheet name="Employee" sheetId="7" r:id="rId4"/>
+    <sheet name="Vacancy" sheetId="8" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <t>Username</t>
   </si>
@@ -153,6 +154,30 @@
   </si>
   <si>
     <t>Current and Past Employees</t>
+  </si>
+  <si>
+    <t>Vacancy</t>
+  </si>
+  <si>
+    <t>Hiring Manager</t>
+  </si>
+  <si>
+    <t>Tester</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Sales IT</t>
+  </si>
+  <si>
+    <t>Nguyễn Bách</t>
+  </si>
+  <si>
+    <t>Nguyễn Quân</t>
+  </si>
+  <si>
+    <t>Closed</t>
   </si>
 </sst>
 </file>
@@ -777,4 +802,65 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E6F5BA6-9A10-48D3-851F-CB3166AA38AB}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="10.8984375" customWidth="1"/>
+    <col min="3" max="3" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix and reffactor with codex :v
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Datadriven-OrangeHrm.xlsx
+++ b/src/test/resources/data/Datadriven-OrangeHrm.xlsx
@@ -680,187 +680,234 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F35673-FDC9-419A-9CAF-7B580C323A56}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{39F35673-FDC9-419A-9CAF-7B580C323A56}">
+  <ns0:dimension ref="A1:D4"/>
+  <ns0:sheetFormatPr defaultRowHeight="13.8" ns3:dyDescent="0.25"/>
+  <ns0:cols>
+    <ns0:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A1" t="s">
+        <ns0:v>16</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" t="s">
+        <ns0:v>17</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" t="s">
+        <ns0:v>18</ns0:v>
+      </ns0:c>
+      <ns0:c r="D1" t="str">
+        <ns0:v>expectedFound</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="C2" t="s">
+        <ns0:v>19</ns0:v>
+      </ns0:c>
+      <ns0:c r="D2" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A3" t="s">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" t="s">
+        <ns0:v>21</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" t="s">
+        <ns0:v>22</ns0:v>
+      </ns0:c>
+      <ns0:c r="D3" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" spans="1:3" ns3:dyDescent="0.25">
+      <ns0:c r="A4" t="s">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF2A67B0-D40E-47CE-8D8C-FABDD5073471}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="21.8984375" customWidth="1"/>
-    <col min="3" max="3" width="18.69921875" customWidth="1"/>
-    <col min="4" max="4" width="24.19921875" customWidth="1"/>
-    <col min="5" max="5" width="24.296875" customWidth="1"/>
-    <col min="7" max="7" width="19.296875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="D2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{EF2A67B0-D40E-47CE-8D8C-FABDD5073471}">
+  <ns0:dimension ref="A1:H5"/>
+  <ns0:sheetFormatPr defaultRowHeight="13.8" ns3:dyDescent="0.25"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="21.8984375" customWidth="1"/>
+    <ns0:col min="3" max="3" width="18.69921875" customWidth="1"/>
+    <ns0:col min="4" max="4" width="24.19921875" customWidth="1"/>
+    <ns0:col min="5" max="5" width="24.296875" customWidth="1"/>
+    <ns0:col min="7" max="7" width="19.296875" customWidth="1"/>
+    <ns0:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:7" ns3:dyDescent="0.25">
+      <ns0:c r="A1" t="s">
+        <ns0:v>16</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="D1" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="E1" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="F1" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="G1" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="H1" t="str">
+        <ns0:v>expectedFound</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:7" ns3:dyDescent="0.25">
+      <ns0:c r="A2" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="1"/>
+      <ns0:c r="D2" t="s">
+        <ns0:v>36</ns0:v>
+      </ns0:c>
+      <ns0:c r="H2" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" spans="1:7" ns3:dyDescent="0.25">
+      <ns0:c r="B3" s="1" t="s">
+        <ns0:v>31</ns0:v>
+      </ns0:c>
+      <ns0:c r="D3" t="s">
+        <ns0:v>33</ns0:v>
+      </ns0:c>
+      <ns0:c r="H3" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" spans="1:7" ns3:dyDescent="0.25">
+      <ns0:c r="C4" t="s">
+        <ns0:v>32</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" t="s">
+        <ns0:v>33</ns0:v>
+      </ns0:c>
+      <ns0:c r="H4" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" spans="1:7" ns3:dyDescent="0.25">
+      <ns0:c r="C5" t="s">
+        <ns0:v>32</ns0:v>
+      </ns0:c>
+      <ns0:c r="D5" t="s">
+        <ns0:v>33</ns0:v>
+      </ns0:c>
+      <ns0:c r="E5" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="F5" t="s">
+        <ns0:v>34</ns0:v>
+      </ns0:c>
+      <ns0:c r="G5" t="s">
+        <ns0:v>35</ns0:v>
+      </ns0:c>
+      <ns0:c r="H5" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:phoneticPr fontId="1" type="noConversion"/>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E6F5BA6-9A10-48D3-851F-CB3166AA38AB}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="10.8984375" customWidth="1"/>
-    <col min="3" max="3" width="17.5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8E6F5BA6-9A10-48D3-851F-CB3166AA38AB}">
+  <ns0:dimension ref="A1:E5"/>
+  <ns0:sheetFormatPr defaultRowHeight="13.8" ns3:dyDescent="0.25"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="12" customWidth="1"/>
+    <ns0:col min="2" max="2" width="10.8984375" customWidth="1"/>
+    <ns0:col min="3" max="3" width="17.5" customWidth="1"/>
+    <ns0:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:4" ns3:dyDescent="0.25">
+      <ns0:c r="A1" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" t="s">
+        <ns0:v>38</ns0:v>
+      </ns0:c>
+      <ns0:c r="D1" t="s">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="E1" t="str">
+        <ns0:v>expectedFound</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:4" ns3:dyDescent="0.25">
+      <ns0:c r="A2" t="s">
+        <ns0:v>34</ns0:v>
+      </ns0:c>
+      <ns0:c r="E2" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" spans="1:4" ns3:dyDescent="0.25">
+      <ns0:c r="B3" t="s">
+        <ns0:v>39</ns0:v>
+      </ns0:c>
+      <ns0:c r="E3" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" spans="1:4" ns3:dyDescent="0.25">
+      <ns0:c r="C4" t="s">
+        <ns0:v>42</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" t="s">
+        <ns0:v>44</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" spans="1:4" ns3:dyDescent="0.25">
+      <ns0:c r="A5" t="s">
+        <ns0:v>41</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" t="s">
+        <ns0:v>41</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" t="s">
+        <ns0:v>43</ns0:v>
+      </ns0:c>
+      <ns0:c r="D5" t="s">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="E5" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
</xml_diff>